<commit_message>
itinerary details WIP 2
</commit_message>
<xml_diff>
--- a/Template/Itinerary Template 2.xlsx
+++ b/Template/Itinerary Template 2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Smart Travel PC\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Smart Travel PC\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA40E8D-652A-431F-AF09-3818C4AAE6B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B92BD3C-05E8-4877-B70C-EC959582A226}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="675" windowWidth="19935" windowHeight="15525" xr2:uid="{9938E8AA-1AE6-42E8-8E13-4BFD1C760FE9}"/>
+    <workbookView xWindow="780" yWindow="330" windowWidth="16650" windowHeight="15870" xr2:uid="{9938E8AA-1AE6-42E8-8E13-4BFD1C760FE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -730,7 +730,6 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
@@ -739,6 +738,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="9"/>
     </xf>
@@ -760,6 +762,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -886,9 +891,6 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1186,12 +1188,10 @@
     <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1588,22 +1588,22 @@
       <c r="L1" s="152"/>
     </row>
     <row r="2" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="171" t="s">
+      <c r="A2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="171"/>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="68" t="s">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="170">
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="20">
         <v>1029365</v>
       </c>
     </row>
@@ -1611,14 +1611,14 @@
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="17" t="s">
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="16" t="s">
         <v>3</v>
       </c>
       <c r="H3" s="159"/>
@@ -1631,13 +1631,13 @@
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="66" t="s">
+      <c r="B4" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="68"/>
       <c r="G4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1889,8 +1889,8 @@
     </row>
     <row r="21" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="20"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="19"/>
       <c r="D21" s="15" t="s">
         <v>13</v>
       </c>
@@ -2495,8 +2495,8 @@
       <c r="K60" s="95"/>
       <c r="L60" s="95"/>
     </row>
-    <row r="61" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="16"/>
+    <row r="61" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="171"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -2510,11 +2510,11 @@
       <c r="L61" s="2"/>
     </row>
     <row r="62" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="69" t="s">
+      <c r="A62" s="170" t="s">
         <v>19</v>
       </c>
-      <c r="B62" s="69"/>
-      <c r="C62" s="69"/>
+      <c r="B62" s="70"/>
+      <c r="C62" s="70"/>
       <c r="D62" s="149"/>
       <c r="E62" s="149"/>
       <c r="F62" s="149"/>
@@ -2526,9 +2526,9 @@
       <c r="L62" s="149"/>
     </row>
     <row r="63" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="69"/>
-      <c r="B63" s="69"/>
-      <c r="C63" s="69"/>
+      <c r="A63" s="170"/>
+      <c r="B63" s="70"/>
+      <c r="C63" s="70"/>
       <c r="D63" s="150" t="s">
         <v>20</v>
       </c>
@@ -2542,9 +2542,9 @@
       <c r="L63" s="151"/>
     </row>
     <row r="64" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="69"/>
-      <c r="B64" s="69"/>
-      <c r="C64" s="69"/>
+      <c r="A64" s="170"/>
+      <c r="B64" s="70"/>
+      <c r="C64" s="70"/>
       <c r="D64" s="150" t="s">
         <v>21</v>
       </c>
@@ -2558,9 +2558,9 @@
       <c r="L64" s="151"/>
     </row>
     <row r="65" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="69"/>
-      <c r="B65" s="69"/>
-      <c r="C65" s="69"/>
+      <c r="A65" s="170"/>
+      <c r="B65" s="70"/>
+      <c r="C65" s="70"/>
       <c r="D65" s="150" t="s">
         <v>22</v>
       </c>
@@ -2574,9 +2574,9 @@
       <c r="L65" s="151"/>
     </row>
     <row r="66" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="69"/>
-      <c r="B66" s="69"/>
-      <c r="C66" s="69"/>
+      <c r="A66" s="170"/>
+      <c r="B66" s="70"/>
+      <c r="C66" s="70"/>
       <c r="D66" s="150" t="s">
         <v>23</v>
       </c>
@@ -2590,9 +2590,9 @@
       <c r="L66" s="151"/>
     </row>
     <row r="67" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="69"/>
-      <c r="B67" s="69"/>
-      <c r="C67" s="69"/>
+      <c r="A67" s="170"/>
+      <c r="B67" s="70"/>
+      <c r="C67" s="70"/>
       <c r="D67" s="150" t="s">
         <v>24</v>
       </c>
@@ -2606,9 +2606,9 @@
       <c r="L67" s="151"/>
     </row>
     <row r="68" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="69"/>
-      <c r="B68" s="69"/>
-      <c r="C68" s="69"/>
+      <c r="A68" s="170"/>
+      <c r="B68" s="70"/>
+      <c r="C68" s="70"/>
       <c r="D68" s="150" t="s">
         <v>25</v>
       </c>
@@ -2622,9 +2622,9 @@
       <c r="L68" s="151"/>
     </row>
     <row r="69" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="69"/>
-      <c r="B69" s="69"/>
-      <c r="C69" s="69"/>
+      <c r="A69" s="170"/>
+      <c r="B69" s="70"/>
+      <c r="C69" s="70"/>
       <c r="D69" s="150" t="s">
         <v>26</v>
       </c>
@@ -2638,7 +2638,7 @@
       <c r="L69" s="151"/>
     </row>
     <row r="70" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="70"/>
+      <c r="A70" s="170"/>
       <c r="B70" s="70"/>
       <c r="C70" s="70"/>
       <c r="D70" s="166"/>
@@ -2788,48 +2788,48 @@
       <c r="L79" s="89"/>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A80" s="31" t="s">
+      <c r="A80" s="32" t="s">
         <v>31</v>
       </c>
       <c r="B80" s="169"/>
       <c r="C80" s="169"/>
-      <c r="D80" s="32"/>
-      <c r="E80" s="32"/>
-      <c r="F80" s="32"/>
-      <c r="G80" s="32"/>
-      <c r="H80" s="32"/>
-      <c r="I80" s="32"/>
-      <c r="J80" s="32"/>
-      <c r="K80" s="32"/>
-      <c r="L80" s="33"/>
+      <c r="D80" s="33"/>
+      <c r="E80" s="33"/>
+      <c r="F80" s="33"/>
+      <c r="G80" s="33"/>
+      <c r="H80" s="33"/>
+      <c r="I80" s="33"/>
+      <c r="J80" s="33"/>
+      <c r="K80" s="33"/>
+      <c r="L80" s="34"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A81" s="34"/>
-      <c r="B81" s="35"/>
-      <c r="C81" s="35"/>
-      <c r="D81" s="35"/>
-      <c r="E81" s="35"/>
-      <c r="F81" s="35"/>
-      <c r="G81" s="35"/>
-      <c r="H81" s="35"/>
-      <c r="I81" s="35"/>
-      <c r="J81" s="35"/>
-      <c r="K81" s="35"/>
-      <c r="L81" s="36"/>
+      <c r="A81" s="35"/>
+      <c r="B81" s="36"/>
+      <c r="C81" s="36"/>
+      <c r="D81" s="36"/>
+      <c r="E81" s="36"/>
+      <c r="F81" s="36"/>
+      <c r="G81" s="36"/>
+      <c r="H81" s="36"/>
+      <c r="I81" s="36"/>
+      <c r="J81" s="36"/>
+      <c r="K81" s="36"/>
+      <c r="L81" s="37"/>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A82" s="55"/>
-      <c r="B82" s="61"/>
-      <c r="C82" s="56"/>
-      <c r="D82" s="52"/>
-      <c r="E82" s="53"/>
-      <c r="F82" s="54"/>
-      <c r="G82" s="52"/>
-      <c r="H82" s="54"/>
-      <c r="I82" s="52"/>
-      <c r="J82" s="53"/>
-      <c r="K82" s="54"/>
-      <c r="L82" s="18" t="s">
+      <c r="A82" s="56"/>
+      <c r="B82" s="62"/>
+      <c r="C82" s="57"/>
+      <c r="D82" s="53"/>
+      <c r="E82" s="54"/>
+      <c r="F82" s="55"/>
+      <c r="G82" s="53"/>
+      <c r="H82" s="55"/>
+      <c r="I82" s="53"/>
+      <c r="J82" s="54"/>
+      <c r="K82" s="55"/>
+      <c r="L82" s="17" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2837,215 +2837,215 @@
       <c r="A83" s="156"/>
       <c r="B83" s="157"/>
       <c r="C83" s="158"/>
-      <c r="D83" s="52"/>
-      <c r="E83" s="53"/>
-      <c r="F83" s="54"/>
-      <c r="G83" s="52"/>
-      <c r="H83" s="54"/>
-      <c r="I83" s="52"/>
-      <c r="J83" s="53"/>
-      <c r="K83" s="54"/>
-      <c r="L83" s="18"/>
+      <c r="D83" s="53"/>
+      <c r="E83" s="54"/>
+      <c r="F83" s="55"/>
+      <c r="G83" s="53"/>
+      <c r="H83" s="55"/>
+      <c r="I83" s="53"/>
+      <c r="J83" s="54"/>
+      <c r="K83" s="55"/>
+      <c r="L83" s="17"/>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A84" s="57"/>
-      <c r="B84" s="62"/>
-      <c r="C84" s="58"/>
-      <c r="D84" s="52"/>
-      <c r="E84" s="53"/>
-      <c r="F84" s="54"/>
-      <c r="G84" s="52"/>
-      <c r="H84" s="54"/>
-      <c r="I84" s="52"/>
-      <c r="J84" s="53"/>
-      <c r="K84" s="54"/>
-      <c r="L84" s="18"/>
+      <c r="A84" s="58"/>
+      <c r="B84" s="63"/>
+      <c r="C84" s="59"/>
+      <c r="D84" s="53"/>
+      <c r="E84" s="54"/>
+      <c r="F84" s="55"/>
+      <c r="G84" s="53"/>
+      <c r="H84" s="55"/>
+      <c r="I84" s="53"/>
+      <c r="J84" s="54"/>
+      <c r="K84" s="55"/>
+      <c r="L84" s="17"/>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A85" s="28" t="s">
+      <c r="A85" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="B85" s="29"/>
-      <c r="C85" s="29"/>
-      <c r="D85" s="29"/>
-      <c r="E85" s="29"/>
-      <c r="F85" s="29"/>
-      <c r="G85" s="29"/>
-      <c r="H85" s="29"/>
-      <c r="I85" s="29"/>
-      <c r="J85" s="29"/>
-      <c r="K85" s="29"/>
-      <c r="L85" s="30"/>
+      <c r="B85" s="30"/>
+      <c r="C85" s="30"/>
+      <c r="D85" s="30"/>
+      <c r="E85" s="30"/>
+      <c r="F85" s="30"/>
+      <c r="G85" s="30"/>
+      <c r="H85" s="30"/>
+      <c r="I85" s="30"/>
+      <c r="J85" s="30"/>
+      <c r="K85" s="30"/>
+      <c r="L85" s="31"/>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A86" s="34"/>
-      <c r="B86" s="35"/>
-      <c r="C86" s="35"/>
-      <c r="D86" s="35"/>
-      <c r="E86" s="35"/>
-      <c r="F86" s="35"/>
-      <c r="G86" s="35"/>
-      <c r="H86" s="35"/>
-      <c r="I86" s="35"/>
-      <c r="J86" s="35"/>
-      <c r="K86" s="35"/>
-      <c r="L86" s="36"/>
+      <c r="A86" s="35"/>
+      <c r="B86" s="36"/>
+      <c r="C86" s="36"/>
+      <c r="D86" s="36"/>
+      <c r="E86" s="36"/>
+      <c r="F86" s="36"/>
+      <c r="G86" s="36"/>
+      <c r="H86" s="36"/>
+      <c r="I86" s="36"/>
+      <c r="J86" s="36"/>
+      <c r="K86" s="36"/>
+      <c r="L86" s="37"/>
     </row>
     <row r="87" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="55"/>
-      <c r="B87" s="61"/>
-      <c r="C87" s="56"/>
-      <c r="D87" s="55"/>
-      <c r="E87" s="56"/>
-      <c r="F87" s="55"/>
-      <c r="G87" s="56"/>
-      <c r="H87" s="59"/>
-      <c r="I87" s="55"/>
-      <c r="J87" s="61"/>
-      <c r="K87" s="56"/>
-      <c r="L87" s="63"/>
+      <c r="A87" s="56"/>
+      <c r="B87" s="62"/>
+      <c r="C87" s="57"/>
+      <c r="D87" s="56"/>
+      <c r="E87" s="57"/>
+      <c r="F87" s="56"/>
+      <c r="G87" s="57"/>
+      <c r="H87" s="60"/>
+      <c r="I87" s="56"/>
+      <c r="J87" s="62"/>
+      <c r="K87" s="57"/>
+      <c r="L87" s="64"/>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" s="156"/>
       <c r="B88" s="157"/>
       <c r="C88" s="158"/>
-      <c r="D88" s="57"/>
-      <c r="E88" s="58"/>
-      <c r="F88" s="57"/>
-      <c r="G88" s="58"/>
-      <c r="H88" s="60"/>
-      <c r="I88" s="57"/>
-      <c r="J88" s="62"/>
-      <c r="K88" s="58"/>
+      <c r="D88" s="58"/>
+      <c r="E88" s="59"/>
+      <c r="F88" s="58"/>
+      <c r="G88" s="59"/>
+      <c r="H88" s="61"/>
+      <c r="I88" s="58"/>
+      <c r="J88" s="63"/>
+      <c r="K88" s="59"/>
       <c r="L88" s="24"/>
     </row>
     <row r="89" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="156"/>
       <c r="B89" s="157"/>
       <c r="C89" s="158"/>
-      <c r="D89" s="55"/>
-      <c r="E89" s="56"/>
-      <c r="F89" s="55"/>
-      <c r="G89" s="56"/>
-      <c r="H89" s="59"/>
-      <c r="I89" s="55"/>
-      <c r="J89" s="61"/>
-      <c r="K89" s="56"/>
-      <c r="L89" s="63"/>
+      <c r="D89" s="56"/>
+      <c r="E89" s="57"/>
+      <c r="F89" s="56"/>
+      <c r="G89" s="57"/>
+      <c r="H89" s="60"/>
+      <c r="I89" s="56"/>
+      <c r="J89" s="62"/>
+      <c r="K89" s="57"/>
+      <c r="L89" s="64"/>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A90" s="57"/>
-      <c r="B90" s="62"/>
-      <c r="C90" s="58"/>
-      <c r="D90" s="57"/>
-      <c r="E90" s="58"/>
-      <c r="F90" s="57"/>
-      <c r="G90" s="58"/>
-      <c r="H90" s="60"/>
-      <c r="I90" s="57"/>
-      <c r="J90" s="62"/>
-      <c r="K90" s="58"/>
+      <c r="A90" s="58"/>
+      <c r="B90" s="63"/>
+      <c r="C90" s="59"/>
+      <c r="D90" s="58"/>
+      <c r="E90" s="59"/>
+      <c r="F90" s="58"/>
+      <c r="G90" s="59"/>
+      <c r="H90" s="61"/>
+      <c r="I90" s="58"/>
+      <c r="J90" s="63"/>
+      <c r="K90" s="59"/>
       <c r="L90" s="24"/>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A91" s="28" t="s">
+      <c r="A91" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B91" s="29"/>
-      <c r="C91" s="30"/>
-      <c r="D91" s="37" t="s">
+      <c r="B91" s="30"/>
+      <c r="C91" s="31"/>
+      <c r="D91" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="E91" s="38"/>
-      <c r="F91" s="39"/>
-      <c r="G91" s="37" t="s">
+      <c r="E91" s="39"/>
+      <c r="F91" s="40"/>
+      <c r="G91" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="H91" s="38"/>
-      <c r="I91" s="38"/>
-      <c r="J91" s="39"/>
-      <c r="K91" s="37" t="s">
+      <c r="H91" s="39"/>
+      <c r="I91" s="39"/>
+      <c r="J91" s="40"/>
+      <c r="K91" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="L91" s="39"/>
+      <c r="L91" s="40"/>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A92" s="31"/>
-      <c r="B92" s="32"/>
-      <c r="C92" s="33"/>
-      <c r="D92" s="40"/>
-      <c r="E92" s="41"/>
-      <c r="F92" s="42"/>
-      <c r="G92" s="40"/>
-      <c r="H92" s="41"/>
-      <c r="I92" s="41"/>
-      <c r="J92" s="42"/>
-      <c r="K92" s="40"/>
-      <c r="L92" s="42"/>
+      <c r="A92" s="32"/>
+      <c r="B92" s="33"/>
+      <c r="C92" s="34"/>
+      <c r="D92" s="41"/>
+      <c r="E92" s="42"/>
+      <c r="F92" s="43"/>
+      <c r="G92" s="41"/>
+      <c r="H92" s="42"/>
+      <c r="I92" s="42"/>
+      <c r="J92" s="43"/>
+      <c r="K92" s="41"/>
+      <c r="L92" s="43"/>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A93" s="31"/>
-      <c r="B93" s="32"/>
-      <c r="C93" s="33"/>
-      <c r="D93" s="37" t="s">
+      <c r="A93" s="32"/>
+      <c r="B93" s="33"/>
+      <c r="C93" s="34"/>
+      <c r="D93" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="E93" s="38"/>
-      <c r="F93" s="39"/>
-      <c r="G93" s="37" t="s">
+      <c r="E93" s="39"/>
+      <c r="F93" s="40"/>
+      <c r="G93" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="H93" s="38"/>
-      <c r="I93" s="38"/>
-      <c r="J93" s="39"/>
-      <c r="K93" s="37" t="s">
+      <c r="H93" s="39"/>
+      <c r="I93" s="39"/>
+      <c r="J93" s="40"/>
+      <c r="K93" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="L93" s="39"/>
+      <c r="L93" s="40"/>
     </row>
     <row r="94" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="34"/>
-      <c r="B94" s="35"/>
-      <c r="C94" s="36"/>
-      <c r="D94" s="40"/>
-      <c r="E94" s="41"/>
-      <c r="F94" s="42"/>
-      <c r="G94" s="40"/>
-      <c r="H94" s="41"/>
-      <c r="I94" s="41"/>
-      <c r="J94" s="42"/>
-      <c r="K94" s="40"/>
-      <c r="L94" s="42"/>
+      <c r="A94" s="35"/>
+      <c r="B94" s="36"/>
+      <c r="C94" s="37"/>
+      <c r="D94" s="41"/>
+      <c r="E94" s="42"/>
+      <c r="F94" s="43"/>
+      <c r="G94" s="41"/>
+      <c r="H94" s="42"/>
+      <c r="I94" s="42"/>
+      <c r="J94" s="43"/>
+      <c r="K94" s="41"/>
+      <c r="L94" s="43"/>
     </row>
     <row r="95" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="43" t="s">
+      <c r="A95" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="B95" s="44"/>
-      <c r="C95" s="44"/>
-      <c r="D95" s="44"/>
-      <c r="E95" s="44"/>
-      <c r="F95" s="44"/>
-      <c r="G95" s="44"/>
-      <c r="H95" s="44"/>
-      <c r="I95" s="44"/>
-      <c r="J95" s="44"/>
-      <c r="K95" s="44"/>
-      <c r="L95" s="45"/>
+      <c r="B95" s="45"/>
+      <c r="C95" s="45"/>
+      <c r="D95" s="45"/>
+      <c r="E95" s="45"/>
+      <c r="F95" s="45"/>
+      <c r="G95" s="45"/>
+      <c r="H95" s="45"/>
+      <c r="I95" s="45"/>
+      <c r="J95" s="45"/>
+      <c r="K95" s="45"/>
+      <c r="L95" s="46"/>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A96" s="46"/>
-      <c r="B96" s="47"/>
-      <c r="C96" s="47"/>
-      <c r="D96" s="47"/>
-      <c r="E96" s="47"/>
-      <c r="F96" s="47"/>
-      <c r="G96" s="47"/>
-      <c r="H96" s="47"/>
-      <c r="I96" s="47"/>
-      <c r="J96" s="47"/>
-      <c r="K96" s="47"/>
-      <c r="L96" s="48"/>
+      <c r="A96" s="47"/>
+      <c r="B96" s="48"/>
+      <c r="C96" s="48"/>
+      <c r="D96" s="48"/>
+      <c r="E96" s="48"/>
+      <c r="F96" s="48"/>
+      <c r="G96" s="48"/>
+      <c r="H96" s="48"/>
+      <c r="I96" s="48"/>
+      <c r="J96" s="48"/>
+      <c r="K96" s="48"/>
+      <c r="L96" s="49"/>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" s="153"/>
@@ -3062,36 +3062,36 @@
       <c r="L97" s="155"/>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A98" s="49" t="s">
+      <c r="A98" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="B98" s="50"/>
-      <c r="C98" s="50"/>
-      <c r="D98" s="50"/>
-      <c r="E98" s="50"/>
-      <c r="F98" s="50"/>
-      <c r="G98" s="50"/>
-      <c r="H98" s="50"/>
-      <c r="I98" s="50"/>
-      <c r="J98" s="50"/>
-      <c r="K98" s="50"/>
-      <c r="L98" s="51"/>
+      <c r="B98" s="51"/>
+      <c r="C98" s="51"/>
+      <c r="D98" s="51"/>
+      <c r="E98" s="51"/>
+      <c r="F98" s="51"/>
+      <c r="G98" s="51"/>
+      <c r="H98" s="51"/>
+      <c r="I98" s="51"/>
+      <c r="J98" s="51"/>
+      <c r="K98" s="51"/>
+      <c r="L98" s="52"/>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A99" s="49" t="s">
+      <c r="A99" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="B99" s="50"/>
-      <c r="C99" s="50"/>
-      <c r="D99" s="50"/>
-      <c r="E99" s="50"/>
-      <c r="F99" s="50"/>
-      <c r="G99" s="50"/>
-      <c r="H99" s="50"/>
-      <c r="I99" s="50"/>
-      <c r="J99" s="50"/>
-      <c r="K99" s="50"/>
-      <c r="L99" s="51"/>
+      <c r="B99" s="51"/>
+      <c r="C99" s="51"/>
+      <c r="D99" s="51"/>
+      <c r="E99" s="51"/>
+      <c r="F99" s="51"/>
+      <c r="G99" s="51"/>
+      <c r="H99" s="51"/>
+      <c r="I99" s="51"/>
+      <c r="J99" s="51"/>
+      <c r="K99" s="51"/>
+      <c r="L99" s="52"/>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="21" t="s">

</xml_diff>